<commit_message>
Refresh stock closing prices
</commit_message>
<xml_diff>
--- a/outputs/stock_closing_prices.xlsx
+++ b/outputs/stock_closing_prices.xlsx
@@ -454,77 +454,77 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>2026-09-07 Close</t>
+          <t>2026-09-08 Close</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>2026-09-07 Change</t>
+          <t>2026-09-08 Change</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>2026-09-07 Change %</t>
+          <t>2026-09-08 Change %</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>2026-09-08 Close</t>
+          <t>2026-09-09 Close</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>2026-09-08 Change</t>
+          <t>2026-09-09 Change</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>2026-09-08 Change %</t>
+          <t>2026-09-09 Change %</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>2026-09-09 Close</t>
+          <t>2026-09-10 Close</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>2026-09-09 Change</t>
+          <t>2026-09-10 Change</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>2026-09-09 Change %</t>
+          <t>2026-09-10 Change %</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>2026-09-10 Close</t>
+          <t>2026-09-11 Close</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>2026-09-10 Change</t>
+          <t>2026-09-11 Change</t>
         </is>
       </c>
       <c r="O1" t="inlineStr">
         <is>
-          <t>2026-09-10 Change %</t>
+          <t>2026-09-11 Change %</t>
         </is>
       </c>
       <c r="P1" t="inlineStr">
         <is>
-          <t>2026-09-11 Close</t>
+          <t>2026-09-14 Close</t>
         </is>
       </c>
       <c r="Q1" t="inlineStr">
         <is>
-          <t>2026-09-11 Change</t>
+          <t>2026-09-14 Change</t>
         </is>
       </c>
       <c r="R1" t="inlineStr">
         <is>
-          <t>2026-09-11 Change %</t>
+          <t>2026-09-14 Change %</t>
         </is>
       </c>
     </row>
@@ -577,49 +577,49 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>167.6</v>
+        <v>164.9</v>
       </c>
       <c r="E3" t="n">
-        <v>0.9</v>
+        <v>-2.7</v>
       </c>
       <c r="F3" t="n">
-        <v>0.54</v>
+        <v>-1.61</v>
       </c>
       <c r="G3" t="n">
-        <v>164.9</v>
+        <v>166</v>
       </c>
       <c r="H3" t="n">
-        <v>-2.7</v>
+        <v>1.1</v>
       </c>
       <c r="I3" t="n">
-        <v>-1.61</v>
+        <v>0.67</v>
       </c>
       <c r="J3" t="n">
-        <v>166</v>
+        <v>164.7</v>
       </c>
       <c r="K3" t="n">
-        <v>1.1</v>
+        <v>-1.3</v>
       </c>
       <c r="L3" t="n">
-        <v>0.67</v>
+        <v>-0.78</v>
       </c>
       <c r="M3" t="n">
-        <v>164.7</v>
+        <v>163.3</v>
       </c>
       <c r="N3" t="n">
-        <v>-1.3</v>
+        <v>-1.4</v>
       </c>
       <c r="O3" t="n">
-        <v>-0.78</v>
+        <v>-0.85</v>
       </c>
       <c r="P3" t="n">
-        <v>164.7</v>
+        <v>163.3</v>
       </c>
       <c r="Q3" t="n">
-        <v>-1.3</v>
+        <v>-1.4</v>
       </c>
       <c r="R3" t="n">
-        <v>-0.78</v>
+        <v>-0.85</v>
       </c>
     </row>
     <row r="4">
@@ -639,49 +639,49 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>239.6</v>
+        <v>239.4</v>
       </c>
       <c r="E4" t="n">
-        <v>2.2</v>
+        <v>-0.2</v>
       </c>
       <c r="F4" t="n">
-        <v>0.93</v>
+        <v>-0.08</v>
       </c>
       <c r="G4" t="n">
-        <v>239.4</v>
+        <v>242.6</v>
       </c>
       <c r="H4" t="n">
-        <v>-0.2</v>
+        <v>3.2</v>
       </c>
       <c r="I4" t="n">
-        <v>-0.08</v>
+        <v>1.34</v>
       </c>
       <c r="J4" t="n">
-        <v>242.6</v>
+        <v>241.8</v>
       </c>
       <c r="K4" t="n">
-        <v>3.2</v>
+        <v>-0.8</v>
       </c>
       <c r="L4" t="n">
-        <v>1.34</v>
+        <v>-0.33</v>
       </c>
       <c r="M4" t="n">
         <v>241.8</v>
       </c>
       <c r="N4" t="n">
-        <v>-0.8</v>
+        <v>0</v>
       </c>
       <c r="O4" t="n">
-        <v>-0.33</v>
+        <v>0</v>
       </c>
       <c r="P4" t="n">
         <v>241.8</v>
       </c>
       <c r="Q4" t="n">
-        <v>-0.8</v>
+        <v>0</v>
       </c>
       <c r="R4" t="n">
-        <v>-0.33</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -701,49 +701,49 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>6.38</v>
+        <v>6.3</v>
       </c>
       <c r="E5" t="n">
-        <v>-0.16</v>
+        <v>-0.08</v>
       </c>
       <c r="F5" t="n">
-        <v>-2.45</v>
+        <v>-1.25</v>
       </c>
       <c r="G5" t="n">
         <v>6.3</v>
       </c>
       <c r="H5" t="n">
-        <v>-0.08</v>
+        <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>-1.25</v>
+        <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>6.3</v>
+        <v>6.38</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>0.08</v>
       </c>
       <c r="L5" t="n">
-        <v>0</v>
+        <v>1.27</v>
       </c>
       <c r="M5" t="n">
-        <v>6.38</v>
+        <v>6.36</v>
       </c>
       <c r="N5" t="n">
-        <v>0.08</v>
+        <v>-0.02</v>
       </c>
       <c r="O5" t="n">
-        <v>1.27</v>
+        <v>-0.31</v>
       </c>
       <c r="P5" t="n">
-        <v>6.38</v>
+        <v>6.36</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.08</v>
+        <v>-0.02</v>
       </c>
       <c r="R5" t="n">
-        <v>1.27</v>
+        <v>-0.31</v>
       </c>
     </row>
     <row r="6">
@@ -766,46 +766,46 @@
         <v>7.51</v>
       </c>
       <c r="E6" t="n">
-        <v>-0.19</v>
+        <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>-2.47</v>
+        <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>7.51</v>
+        <v>7.55</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>0.04</v>
       </c>
       <c r="I6" t="n">
-        <v>0</v>
+        <v>0.53</v>
       </c>
       <c r="J6" t="n">
-        <v>7.55</v>
+        <v>7.61</v>
       </c>
       <c r="K6" t="n">
-        <v>0.04</v>
+        <v>0.06</v>
       </c>
       <c r="L6" t="n">
-        <v>0.53</v>
+        <v>0.79</v>
       </c>
       <c r="M6" t="n">
         <v>7.61</v>
       </c>
       <c r="N6" t="n">
-        <v>0.06</v>
+        <v>0</v>
       </c>
       <c r="O6" t="n">
-        <v>0.79</v>
+        <v>0</v>
       </c>
       <c r="P6" t="n">
         <v>7.61</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.06</v>
+        <v>0</v>
       </c>
       <c r="R6" t="n">
-        <v>0.79</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -825,49 +825,49 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>5.95</v>
+        <v>5.88</v>
       </c>
       <c r="E7" t="n">
-        <v>-0.12</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="F7" t="n">
-        <v>-1.98</v>
+        <v>-1.18</v>
       </c>
       <c r="G7" t="n">
-        <v>5.88</v>
+        <v>5.91</v>
       </c>
       <c r="H7" t="n">
-        <v>-0.07000000000000001</v>
+        <v>0.03</v>
       </c>
       <c r="I7" t="n">
-        <v>-1.18</v>
+        <v>0.51</v>
       </c>
       <c r="J7" t="n">
-        <v>5.91</v>
+        <v>5.97</v>
       </c>
       <c r="K7" t="n">
-        <v>0.03</v>
+        <v>0.06</v>
       </c>
       <c r="L7" t="n">
-        <v>0.51</v>
+        <v>1.02</v>
       </c>
       <c r="M7" t="n">
-        <v>5.97</v>
+        <v>6.05</v>
       </c>
       <c r="N7" t="n">
-        <v>0.06</v>
+        <v>0.08</v>
       </c>
       <c r="O7" t="n">
-        <v>1.02</v>
+        <v>1.34</v>
       </c>
       <c r="P7" t="n">
-        <v>5.97</v>
+        <v>6.05</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.06</v>
+        <v>0.08</v>
       </c>
       <c r="R7" t="n">
-        <v>1.02</v>
+        <v>1.34</v>
       </c>
     </row>
     <row r="8">
@@ -887,49 +887,49 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>9.529999999999999</v>
+        <v>9.56</v>
       </c>
       <c r="E8" t="n">
-        <v>-0.23</v>
+        <v>0.03</v>
       </c>
       <c r="F8" t="n">
-        <v>-2.36</v>
+        <v>0.31</v>
       </c>
       <c r="G8" t="n">
-        <v>9.56</v>
+        <v>9.609999999999999</v>
       </c>
       <c r="H8" t="n">
-        <v>0.03</v>
+        <v>0.05</v>
       </c>
       <c r="I8" t="n">
-        <v>0.31</v>
+        <v>0.52</v>
       </c>
       <c r="J8" t="n">
-        <v>9.609999999999999</v>
+        <v>9.77</v>
       </c>
       <c r="K8" t="n">
-        <v>0.05</v>
+        <v>0.16</v>
       </c>
       <c r="L8" t="n">
-        <v>0.52</v>
+        <v>1.66</v>
       </c>
       <c r="M8" t="n">
-        <v>9.77</v>
+        <v>9.75</v>
       </c>
       <c r="N8" t="n">
-        <v>0.16</v>
+        <v>-0.02</v>
       </c>
       <c r="O8" t="n">
-        <v>1.66</v>
+        <v>-0.2</v>
       </c>
       <c r="P8" t="n">
-        <v>9.77</v>
+        <v>9.75</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.16</v>
+        <v>-0.02</v>
       </c>
       <c r="R8" t="n">
-        <v>1.66</v>
+        <v>-0.2</v>
       </c>
     </row>
     <row r="9">
@@ -949,49 +949,49 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>7.88</v>
+        <v>7.86</v>
       </c>
       <c r="E9" t="n">
-        <v>-0.11</v>
+        <v>-0.02</v>
       </c>
       <c r="F9" t="n">
-        <v>-1.38</v>
+        <v>-0.25</v>
       </c>
       <c r="G9" t="n">
-        <v>7.86</v>
+        <v>7.89</v>
       </c>
       <c r="H9" t="n">
-        <v>-0.02</v>
+        <v>0.03</v>
       </c>
       <c r="I9" t="n">
-        <v>-0.25</v>
+        <v>0.38</v>
       </c>
       <c r="J9" t="n">
-        <v>7.89</v>
+        <v>8.06</v>
       </c>
       <c r="K9" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="L9" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="M9" t="n">
+        <v>8.09</v>
+      </c>
+      <c r="N9" t="n">
         <v>0.03</v>
       </c>
-      <c r="L9" t="n">
-        <v>0.38</v>
-      </c>
-      <c r="M9" t="n">
-        <v>8.06</v>
-      </c>
-      <c r="N9" t="n">
-        <v>0.17</v>
-      </c>
       <c r="O9" t="n">
-        <v>2.15</v>
+        <v>0.37</v>
       </c>
       <c r="P9" t="n">
-        <v>8.06</v>
+        <v>8.09</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.17</v>
+        <v>0.03</v>
       </c>
       <c r="R9" t="n">
-        <v>2.15</v>
+        <v>0.37</v>
       </c>
     </row>
     <row r="10">
@@ -1014,46 +1014,46 @@
         <v>51.9</v>
       </c>
       <c r="E10" t="n">
-        <v>-1.45</v>
+        <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>-2.72</v>
+        <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>51.9</v>
+        <v>51.85</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>-0.05</v>
       </c>
       <c r="I10" t="n">
-        <v>0</v>
+        <v>-0.1</v>
       </c>
       <c r="J10" t="n">
-        <v>51.85</v>
+        <v>52.15</v>
       </c>
       <c r="K10" t="n">
-        <v>-0.05</v>
+        <v>0.3</v>
       </c>
       <c r="L10" t="n">
-        <v>-0.1</v>
+        <v>0.58</v>
       </c>
       <c r="M10" t="n">
-        <v>52.15</v>
+        <v>51.95</v>
       </c>
       <c r="N10" t="n">
-        <v>0.3</v>
+        <v>-0.2</v>
       </c>
       <c r="O10" t="n">
-        <v>0.58</v>
+        <v>-0.38</v>
       </c>
       <c r="P10" t="n">
-        <v>52.15</v>
+        <v>51.95</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.3</v>
+        <v>-0.2</v>
       </c>
       <c r="R10" t="n">
-        <v>0.58</v>
+        <v>-0.38</v>
       </c>
     </row>
     <row r="11">
@@ -1073,49 +1073,49 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>4.72</v>
+        <v>4.91</v>
       </c>
       <c r="E11" t="n">
-        <v>-0.07000000000000001</v>
+        <v>0.19</v>
       </c>
       <c r="F11" t="n">
-        <v>-1.46</v>
+        <v>4.03</v>
       </c>
       <c r="G11" t="n">
-        <v>4.91</v>
+        <v>4.92</v>
       </c>
       <c r="H11" t="n">
-        <v>0.19</v>
+        <v>0.01</v>
       </c>
       <c r="I11" t="n">
-        <v>4.03</v>
+        <v>0.2</v>
       </c>
       <c r="J11" t="n">
-        <v>4.92</v>
+        <v>4.84</v>
       </c>
       <c r="K11" t="n">
-        <v>0.01</v>
+        <v>-0.08</v>
       </c>
       <c r="L11" t="n">
-        <v>0.2</v>
+        <v>-1.63</v>
       </c>
       <c r="M11" t="n">
-        <v>4.84</v>
+        <v>4.78</v>
       </c>
       <c r="N11" t="n">
-        <v>-0.08</v>
+        <v>-0.06</v>
       </c>
       <c r="O11" t="n">
-        <v>-1.63</v>
+        <v>-1.24</v>
       </c>
       <c r="P11" t="n">
-        <v>4.84</v>
+        <v>4.78</v>
       </c>
       <c r="Q11" t="n">
-        <v>-0.08</v>
+        <v>-0.06</v>
       </c>
       <c r="R11" t="n">
-        <v>-1.63</v>
+        <v>-1.24</v>
       </c>
     </row>
     <row r="12">
@@ -1135,49 +1135,49 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>9.960000000000001</v>
+        <v>10.35</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.2</v>
+        <v>0.39</v>
       </c>
       <c r="F12" t="n">
-        <v>-1.97</v>
+        <v>3.92</v>
       </c>
       <c r="G12" t="n">
-        <v>10.35</v>
+        <v>10.43</v>
       </c>
       <c r="H12" t="n">
-        <v>0.39</v>
+        <v>0.08</v>
       </c>
       <c r="I12" t="n">
-        <v>3.92</v>
+        <v>0.77</v>
       </c>
       <c r="J12" t="n">
-        <v>10.43</v>
+        <v>10.09</v>
       </c>
       <c r="K12" t="n">
-        <v>0.08</v>
+        <v>-0.34</v>
       </c>
       <c r="L12" t="n">
-        <v>0.77</v>
+        <v>-3.26</v>
       </c>
       <c r="M12" t="n">
-        <v>10.09</v>
+        <v>9.98</v>
       </c>
       <c r="N12" t="n">
-        <v>-0.34</v>
+        <v>-0.11</v>
       </c>
       <c r="O12" t="n">
-        <v>-3.26</v>
+        <v>-1.09</v>
       </c>
       <c r="P12" t="n">
-        <v>10.09</v>
+        <v>9.98</v>
       </c>
       <c r="Q12" t="n">
-        <v>-0.34</v>
+        <v>-0.11</v>
       </c>
       <c r="R12" t="n">
-        <v>-3.26</v>
+        <v>-1.09</v>
       </c>
     </row>
     <row r="13">
@@ -1197,49 +1197,49 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>24.88</v>
+        <v>25.86</v>
       </c>
       <c r="E13" t="n">
-        <v>-0.18</v>
+        <v>0.98</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.72</v>
+        <v>3.94</v>
       </c>
       <c r="G13" t="n">
-        <v>25.86</v>
+        <v>25.82</v>
       </c>
       <c r="H13" t="n">
-        <v>0.98</v>
+        <v>-0.04</v>
       </c>
       <c r="I13" t="n">
-        <v>3.94</v>
+        <v>-0.15</v>
       </c>
       <c r="J13" t="n">
-        <v>25.82</v>
+        <v>25.02</v>
       </c>
       <c r="K13" t="n">
-        <v>-0.04</v>
+        <v>-0.8</v>
       </c>
       <c r="L13" t="n">
-        <v>-0.15</v>
+        <v>-3.1</v>
       </c>
       <c r="M13" t="n">
-        <v>25.02</v>
+        <v>24.38</v>
       </c>
       <c r="N13" t="n">
-        <v>-0.8</v>
+        <v>-0.64</v>
       </c>
       <c r="O13" t="n">
-        <v>-3.1</v>
+        <v>-2.56</v>
       </c>
       <c r="P13" t="n">
-        <v>25.02</v>
+        <v>24.38</v>
       </c>
       <c r="Q13" t="n">
-        <v>-0.8</v>
+        <v>-0.64</v>
       </c>
       <c r="R13" t="n">
-        <v>-3.1</v>
+        <v>-2.56</v>
       </c>
     </row>
     <row r="14">
@@ -1259,49 +1259,49 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>1.97</v>
+        <v>2</v>
       </c>
       <c r="E14" t="n">
-        <v>-0.01</v>
+        <v>0.03</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.51</v>
+        <v>1.52</v>
       </c>
       <c r="G14" t="n">
-        <v>2</v>
+        <v>2.05</v>
       </c>
       <c r="H14" t="n">
-        <v>0.03</v>
+        <v>0.05</v>
       </c>
       <c r="I14" t="n">
-        <v>1.52</v>
+        <v>2.5</v>
       </c>
       <c r="J14" t="n">
-        <v>2.05</v>
+        <v>2.02</v>
       </c>
       <c r="K14" t="n">
-        <v>0.05</v>
+        <v>-0.03</v>
       </c>
       <c r="L14" t="n">
-        <v>2.5</v>
+        <v>-1.46</v>
       </c>
       <c r="M14" t="n">
-        <v>2.02</v>
+        <v>1.98</v>
       </c>
       <c r="N14" t="n">
-        <v>-0.03</v>
+        <v>-0.04</v>
       </c>
       <c r="O14" t="n">
-        <v>-1.46</v>
+        <v>-1.98</v>
       </c>
       <c r="P14" t="n">
-        <v>2.02</v>
+        <v>1.98</v>
       </c>
       <c r="Q14" t="n">
-        <v>-0.03</v>
+        <v>-0.04</v>
       </c>
       <c r="R14" t="n">
-        <v>-1.46</v>
+        <v>-1.98</v>
       </c>
     </row>
     <row r="15">
@@ -1321,16 +1321,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>5.43</v>
+        <v>5.41</v>
       </c>
       <c r="E15" t="n">
-        <v>0.06</v>
+        <v>-0.02</v>
       </c>
       <c r="F15" t="n">
-        <v>1.12</v>
+        <v>-0.37</v>
       </c>
       <c r="G15" t="n">
-        <v>5.41</v>
+        <v>5.39</v>
       </c>
       <c r="H15" t="n">
         <v>-0.02</v>
@@ -1339,31 +1339,31 @@
         <v>-0.37</v>
       </c>
       <c r="J15" t="n">
-        <v>5.39</v>
+        <v>5.23</v>
       </c>
       <c r="K15" t="n">
-        <v>-0.02</v>
+        <v>-0.16</v>
       </c>
       <c r="L15" t="n">
-        <v>-0.37</v>
+        <v>-2.97</v>
       </c>
       <c r="M15" t="n">
-        <v>5.23</v>
+        <v>5.29</v>
       </c>
       <c r="N15" t="n">
-        <v>-0.16</v>
+        <v>0.06</v>
       </c>
       <c r="O15" t="n">
-        <v>-2.97</v>
+        <v>1.15</v>
       </c>
       <c r="P15" t="n">
-        <v>5.23</v>
+        <v>5.29</v>
       </c>
       <c r="Q15" t="n">
-        <v>-0.16</v>
+        <v>0.06</v>
       </c>
       <c r="R15" t="n">
-        <v>-2.97</v>
+        <v>1.15</v>
       </c>
     </row>
     <row r="16">
@@ -1383,49 +1383,49 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>4.41</v>
+        <v>4.46</v>
       </c>
       <c r="E16" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="F16" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="G16" t="n">
+        <v>4.45</v>
+      </c>
+      <c r="H16" t="n">
+        <v>-0.01</v>
+      </c>
+      <c r="I16" t="n">
+        <v>-0.22</v>
+      </c>
+      <c r="J16" t="n">
+        <v>4.43</v>
+      </c>
+      <c r="K16" t="n">
         <v>-0.02</v>
       </c>
-      <c r="F16" t="n">
+      <c r="L16" t="n">
         <v>-0.45</v>
       </c>
-      <c r="G16" t="n">
-        <v>4.46</v>
-      </c>
-      <c r="H16" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="I16" t="n">
-        <v>1.13</v>
-      </c>
-      <c r="J16" t="n">
-        <v>4.45</v>
-      </c>
-      <c r="K16" t="n">
-        <v>-0.01</v>
-      </c>
-      <c r="L16" t="n">
-        <v>-0.22</v>
-      </c>
       <c r="M16" t="n">
-        <v>4.43</v>
+        <v>4.44</v>
       </c>
       <c r="N16" t="n">
-        <v>-0.02</v>
+        <v>0.01</v>
       </c>
       <c r="O16" t="n">
-        <v>-0.45</v>
+        <v>0.23</v>
       </c>
       <c r="P16" t="n">
-        <v>4.43</v>
+        <v>4.44</v>
       </c>
       <c r="Q16" t="n">
-        <v>-0.02</v>
+        <v>0.01</v>
       </c>
       <c r="R16" t="n">
-        <v>-0.45</v>
+        <v>0.23</v>
       </c>
     </row>
     <row r="17">
@@ -1445,49 +1445,49 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>3.35</v>
+        <v>3.38</v>
       </c>
       <c r="E17" t="n">
-        <v>-0.02</v>
+        <v>0.03</v>
       </c>
       <c r="F17" t="n">
-        <v>-0.59</v>
+        <v>0.9</v>
       </c>
       <c r="G17" t="n">
-        <v>3.38</v>
+        <v>3.42</v>
       </c>
       <c r="H17" t="n">
-        <v>0.03</v>
+        <v>0.04</v>
       </c>
       <c r="I17" t="n">
-        <v>0.9</v>
+        <v>1.18</v>
       </c>
       <c r="J17" t="n">
-        <v>3.42</v>
+        <v>3.41</v>
       </c>
       <c r="K17" t="n">
-        <v>0.04</v>
+        <v>-0.01</v>
       </c>
       <c r="L17" t="n">
-        <v>1.18</v>
+        <v>-0.29</v>
       </c>
       <c r="M17" t="n">
-        <v>3.41</v>
+        <v>3.33</v>
       </c>
       <c r="N17" t="n">
-        <v>-0.01</v>
+        <v>-0.08</v>
       </c>
       <c r="O17" t="n">
-        <v>-0.29</v>
+        <v>-2.35</v>
       </c>
       <c r="P17" t="n">
-        <v>3.41</v>
+        <v>3.33</v>
       </c>
       <c r="Q17" t="n">
-        <v>-0.01</v>
+        <v>-0.08</v>
       </c>
       <c r="R17" t="n">
-        <v>-0.29</v>
+        <v>-2.35</v>
       </c>
     </row>
     <row r="18">
@@ -1507,7 +1507,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>3.16</v>
+        <v>3.15</v>
       </c>
       <c r="E18" t="n">
         <v>-0.01</v>
@@ -1516,40 +1516,40 @@
         <v>-0.32</v>
       </c>
       <c r="G18" t="n">
-        <v>3.15</v>
+        <v>3.13</v>
       </c>
       <c r="H18" t="n">
-        <v>-0.01</v>
+        <v>-0.02</v>
       </c>
       <c r="I18" t="n">
-        <v>-0.32</v>
+        <v>-0.63</v>
       </c>
       <c r="J18" t="n">
-        <v>3.13</v>
+        <v>3.14</v>
       </c>
       <c r="K18" t="n">
-        <v>-0.02</v>
+        <v>0.01</v>
       </c>
       <c r="L18" t="n">
-        <v>-0.63</v>
+        <v>0.32</v>
       </c>
       <c r="M18" t="n">
-        <v>3.14</v>
+        <v>3.11</v>
       </c>
       <c r="N18" t="n">
-        <v>0.01</v>
+        <v>-0.03</v>
       </c>
       <c r="O18" t="n">
-        <v>0.32</v>
+        <v>-0.96</v>
       </c>
       <c r="P18" t="n">
-        <v>3.14</v>
+        <v>3.11</v>
       </c>
       <c r="Q18" t="n">
-        <v>0.01</v>
+        <v>-0.03</v>
       </c>
       <c r="R18" t="n">
-        <v>0.32</v>
+        <v>-0.96</v>
       </c>
     </row>
     <row r="19">
@@ -1569,49 +1569,49 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>56.25</v>
+        <v>55.25</v>
       </c>
       <c r="E19" t="n">
-        <v>-0.9</v>
+        <v>-1</v>
       </c>
       <c r="F19" t="n">
-        <v>-1.57</v>
+        <v>-1.78</v>
       </c>
       <c r="G19" t="n">
-        <v>55.25</v>
+        <v>55.45</v>
       </c>
       <c r="H19" t="n">
-        <v>-1</v>
+        <v>0.2</v>
       </c>
       <c r="I19" t="n">
-        <v>-1.78</v>
+        <v>0.36</v>
       </c>
       <c r="J19" t="n">
-        <v>55.45</v>
+        <v>54.85</v>
       </c>
       <c r="K19" t="n">
-        <v>0.2</v>
+        <v>-0.6</v>
       </c>
       <c r="L19" t="n">
-        <v>0.36</v>
+        <v>-1.08</v>
       </c>
       <c r="M19" t="n">
-        <v>54.85</v>
+        <v>54</v>
       </c>
       <c r="N19" t="n">
-        <v>-0.6</v>
+        <v>-0.85</v>
       </c>
       <c r="O19" t="n">
-        <v>-1.08</v>
+        <v>-1.55</v>
       </c>
       <c r="P19" t="n">
-        <v>54.85</v>
+        <v>54</v>
       </c>
       <c r="Q19" t="n">
-        <v>-0.6</v>
+        <v>-0.85</v>
       </c>
       <c r="R19" t="n">
-        <v>-1.08</v>
+        <v>-1.55</v>
       </c>
     </row>
     <row r="20">
@@ -1631,49 +1631,49 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>30.56</v>
+        <v>29.62</v>
       </c>
       <c r="E20" t="n">
-        <v>-0.34</v>
+        <v>-0.9399999999999999</v>
       </c>
       <c r="F20" t="n">
-        <v>-1.1</v>
+        <v>-3.08</v>
       </c>
       <c r="G20" t="n">
-        <v>29.62</v>
+        <v>29.48</v>
       </c>
       <c r="H20" t="n">
-        <v>-0.9399999999999999</v>
+        <v>-0.14</v>
       </c>
       <c r="I20" t="n">
-        <v>-3.08</v>
+        <v>-0.47</v>
       </c>
       <c r="J20" t="n">
-        <v>29.48</v>
+        <v>30.14</v>
       </c>
       <c r="K20" t="n">
-        <v>-0.14</v>
+        <v>0.66</v>
       </c>
       <c r="L20" t="n">
-        <v>-0.47</v>
+        <v>2.24</v>
       </c>
       <c r="M20" t="n">
-        <v>30.14</v>
+        <v>29.6</v>
       </c>
       <c r="N20" t="n">
-        <v>0.66</v>
+        <v>-0.54</v>
       </c>
       <c r="O20" t="n">
-        <v>2.24</v>
+        <v>-1.79</v>
       </c>
       <c r="P20" t="n">
-        <v>30.14</v>
+        <v>29.6</v>
       </c>
       <c r="Q20" t="n">
-        <v>0.66</v>
+        <v>-0.54</v>
       </c>
       <c r="R20" t="n">
-        <v>2.24</v>
+        <v>-1.79</v>
       </c>
     </row>
     <row r="21">
@@ -1696,46 +1696,46 @@
         <v>4.58</v>
       </c>
       <c r="E21" t="n">
-        <v>-0.08</v>
+        <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>-1.72</v>
+        <v>0</v>
       </c>
       <c r="G21" t="n">
-        <v>4.58</v>
+        <v>4.55</v>
       </c>
       <c r="H21" t="n">
-        <v>0</v>
+        <v>-0.03</v>
       </c>
       <c r="I21" t="n">
-        <v>0</v>
+        <v>-0.66</v>
       </c>
       <c r="J21" t="n">
-        <v>4.55</v>
+        <v>4.61</v>
       </c>
       <c r="K21" t="n">
-        <v>-0.03</v>
+        <v>0.06</v>
       </c>
       <c r="L21" t="n">
-        <v>-0.66</v>
+        <v>1.32</v>
       </c>
       <c r="M21" t="n">
-        <v>4.61</v>
+        <v>4.52</v>
       </c>
       <c r="N21" t="n">
-        <v>0.06</v>
+        <v>-0.09</v>
       </c>
       <c r="O21" t="n">
-        <v>1.32</v>
+        <v>-1.95</v>
       </c>
       <c r="P21" t="n">
-        <v>4.61</v>
+        <v>4.52</v>
       </c>
       <c r="Q21" t="n">
-        <v>0.06</v>
+        <v>-0.09</v>
       </c>
       <c r="R21" t="n">
-        <v>1.32</v>
+        <v>-1.95</v>
       </c>
     </row>
     <row r="22">
@@ -1755,49 +1755,49 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>79.09999999999999</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="E22" t="n">
-        <v>-0.55</v>
+        <v>-0.2</v>
       </c>
       <c r="F22" t="n">
-        <v>-0.6899999999999999</v>
+        <v>-0.25</v>
       </c>
       <c r="G22" t="n">
+        <v>78.95</v>
+      </c>
+      <c r="H22" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="I22" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="J22" t="n">
+        <v>78.84999999999999</v>
+      </c>
+      <c r="K22" t="n">
+        <v>-0.1</v>
+      </c>
+      <c r="L22" t="n">
+        <v>-0.13</v>
+      </c>
+      <c r="M22" t="n">
         <v>78.90000000000001</v>
       </c>
-      <c r="H22" t="n">
-        <v>-0.2</v>
-      </c>
-      <c r="I22" t="n">
-        <v>-0.25</v>
-      </c>
-      <c r="J22" t="n">
-        <v>78.95</v>
-      </c>
-      <c r="K22" t="n">
+      <c r="N22" t="n">
         <v>0.05</v>
       </c>
-      <c r="L22" t="n">
+      <c r="O22" t="n">
         <v>0.06</v>
       </c>
-      <c r="M22" t="n">
-        <v>78.84999999999999</v>
-      </c>
-      <c r="N22" t="n">
-        <v>-0.1</v>
-      </c>
-      <c r="O22" t="n">
-        <v>-0.13</v>
-      </c>
       <c r="P22" t="n">
-        <v>78.84999999999999</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="Q22" t="n">
-        <v>-0.1</v>
+        <v>0.05</v>
       </c>
       <c r="R22" t="n">
-        <v>-0.13</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="23">
@@ -1817,49 +1817,49 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>23.8</v>
+        <v>23.62</v>
       </c>
       <c r="E23" t="n">
-        <v>0.4</v>
+        <v>-0.18</v>
       </c>
       <c r="F23" t="n">
-        <v>1.71</v>
+        <v>-0.76</v>
       </c>
       <c r="G23" t="n">
-        <v>23.62</v>
+        <v>23.48</v>
       </c>
       <c r="H23" t="n">
-        <v>-0.18</v>
+        <v>-0.14</v>
       </c>
       <c r="I23" t="n">
-        <v>-0.76</v>
+        <v>-0.59</v>
       </c>
       <c r="J23" t="n">
-        <v>23.48</v>
+        <v>22.98</v>
       </c>
       <c r="K23" t="n">
-        <v>-0.14</v>
+        <v>-0.5</v>
       </c>
       <c r="L23" t="n">
-        <v>-0.59</v>
+        <v>-2.13</v>
       </c>
       <c r="M23" t="n">
         <v>22.98</v>
       </c>
       <c r="N23" t="n">
-        <v>-0.5</v>
+        <v>0</v>
       </c>
       <c r="O23" t="n">
-        <v>-2.13</v>
+        <v>0</v>
       </c>
       <c r="P23" t="n">
         <v>22.98</v>
       </c>
       <c r="Q23" t="n">
-        <v>-0.5</v>
+        <v>0</v>
       </c>
       <c r="R23" t="n">
-        <v>-2.13</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
@@ -1879,49 +1879,49 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>16.8</v>
+        <v>16.41</v>
       </c>
       <c r="E24" t="n">
-        <v>0.35</v>
+        <v>-0.39</v>
       </c>
       <c r="F24" t="n">
-        <v>2.13</v>
+        <v>-2.32</v>
       </c>
       <c r="G24" t="n">
+        <v>16.94</v>
+      </c>
+      <c r="H24" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="I24" t="n">
+        <v>3.23</v>
+      </c>
+      <c r="J24" t="n">
+        <v>16.74</v>
+      </c>
+      <c r="K24" t="n">
+        <v>-0.2</v>
+      </c>
+      <c r="L24" t="n">
+        <v>-1.18</v>
+      </c>
+      <c r="M24" t="n">
         <v>16.41</v>
       </c>
-      <c r="H24" t="n">
-        <v>-0.39</v>
-      </c>
-      <c r="I24" t="n">
-        <v>-2.32</v>
-      </c>
-      <c r="J24" t="n">
-        <v>16.94</v>
-      </c>
-      <c r="K24" t="n">
-        <v>0.53</v>
-      </c>
-      <c r="L24" t="n">
-        <v>3.23</v>
-      </c>
-      <c r="M24" t="n">
-        <v>16.74</v>
-      </c>
       <c r="N24" t="n">
-        <v>-0.2</v>
+        <v>-0.33</v>
       </c>
       <c r="O24" t="n">
-        <v>-1.18</v>
+        <v>-1.97</v>
       </c>
       <c r="P24" t="n">
-        <v>16.74</v>
+        <v>16.41</v>
       </c>
       <c r="Q24" t="n">
-        <v>-0.2</v>
+        <v>-0.33</v>
       </c>
       <c r="R24" t="n">
-        <v>-1.18</v>
+        <v>-1.97</v>
       </c>
     </row>
     <row r="25">
@@ -1941,49 +1941,49 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>27.5</v>
+        <v>26.92</v>
       </c>
       <c r="E25" t="n">
-        <v>-0.9399999999999999</v>
+        <v>-0.58</v>
       </c>
       <c r="F25" t="n">
-        <v>-3.31</v>
+        <v>-2.11</v>
       </c>
       <c r="G25" t="n">
-        <v>26.92</v>
+        <v>26.38</v>
       </c>
       <c r="H25" t="n">
-        <v>-0.58</v>
+        <v>-0.54</v>
       </c>
       <c r="I25" t="n">
-        <v>-2.11</v>
+        <v>-2.01</v>
       </c>
       <c r="J25" t="n">
-        <v>26.38</v>
+        <v>25.92</v>
       </c>
       <c r="K25" t="n">
-        <v>-0.54</v>
+        <v>-0.46</v>
       </c>
       <c r="L25" t="n">
-        <v>-2.01</v>
+        <v>-1.74</v>
       </c>
       <c r="M25" t="n">
-        <v>25.92</v>
+        <v>26.36</v>
       </c>
       <c r="N25" t="n">
-        <v>-0.46</v>
+        <v>0.44</v>
       </c>
       <c r="O25" t="n">
-        <v>-1.74</v>
+        <v>1.7</v>
       </c>
       <c r="P25" t="n">
-        <v>25.92</v>
+        <v>26.36</v>
       </c>
       <c r="Q25" t="n">
-        <v>-0.46</v>
+        <v>0.44</v>
       </c>
       <c r="R25" t="n">
-        <v>-1.74</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="26">
@@ -2003,49 +2003,49 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>41.16</v>
+        <v>38.2</v>
       </c>
       <c r="E26" t="n">
-        <v>-0.44</v>
+        <v>-2.96</v>
       </c>
       <c r="F26" t="n">
-        <v>-1.06</v>
+        <v>-7.19</v>
       </c>
       <c r="G26" t="n">
-        <v>38.2</v>
+        <v>38.22</v>
       </c>
       <c r="H26" t="n">
-        <v>-2.96</v>
+        <v>0.02</v>
       </c>
       <c r="I26" t="n">
-        <v>-7.19</v>
+        <v>0.05</v>
       </c>
       <c r="J26" t="n">
-        <v>38.22</v>
+        <v>37.48</v>
       </c>
       <c r="K26" t="n">
-        <v>0.02</v>
+        <v>-0.74</v>
       </c>
       <c r="L26" t="n">
-        <v>0.05</v>
+        <v>-1.94</v>
       </c>
       <c r="M26" t="n">
-        <v>37.48</v>
+        <v>35.46</v>
       </c>
       <c r="N26" t="n">
-        <v>-0.74</v>
+        <v>-2.02</v>
       </c>
       <c r="O26" t="n">
-        <v>-1.94</v>
+        <v>-5.39</v>
       </c>
       <c r="P26" t="n">
-        <v>37.48</v>
+        <v>35.46</v>
       </c>
       <c r="Q26" t="n">
-        <v>-0.74</v>
+        <v>-2.02</v>
       </c>
       <c r="R26" t="n">
-        <v>-1.94</v>
+        <v>-5.39</v>
       </c>
     </row>
     <row r="27">
@@ -2065,49 +2065,49 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>438.4</v>
+        <v>435.4</v>
       </c>
       <c r="E27" t="n">
-        <v>-4.4</v>
+        <v>-3</v>
       </c>
       <c r="F27" t="n">
-        <v>-0.99</v>
+        <v>-0.68</v>
       </c>
       <c r="G27" t="n">
-        <v>435.4</v>
+        <v>434</v>
       </c>
       <c r="H27" t="n">
-        <v>-3</v>
+        <v>-1.4</v>
       </c>
       <c r="I27" t="n">
-        <v>-0.68</v>
+        <v>-0.32</v>
       </c>
       <c r="J27" t="n">
-        <v>434</v>
+        <v>425.6</v>
       </c>
       <c r="K27" t="n">
-        <v>-1.4</v>
+        <v>-8.4</v>
       </c>
       <c r="L27" t="n">
-        <v>-0.32</v>
+        <v>-1.94</v>
       </c>
       <c r="M27" t="n">
-        <v>425.6</v>
+        <v>428.4</v>
       </c>
       <c r="N27" t="n">
-        <v>-8.4</v>
+        <v>2.8</v>
       </c>
       <c r="O27" t="n">
-        <v>-1.94</v>
+        <v>0.66</v>
       </c>
       <c r="P27" t="n">
-        <v>425.6</v>
+        <v>428.4</v>
       </c>
       <c r="Q27" t="n">
-        <v>-8.4</v>
+        <v>2.8</v>
       </c>
       <c r="R27" t="n">
-        <v>-1.94</v>
+        <v>0.66</v>
       </c>
     </row>
     <row r="28">
@@ -2127,49 +2127,49 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>109.6</v>
+        <v>109.5</v>
       </c>
       <c r="E28" t="n">
-        <v>-0.5</v>
+        <v>-0.1</v>
       </c>
       <c r="F28" t="n">
-        <v>-0.45</v>
+        <v>-0.09</v>
       </c>
       <c r="G28" t="n">
-        <v>109.5</v>
+        <v>109.8</v>
       </c>
       <c r="H28" t="n">
-        <v>-0.1</v>
+        <v>0.3</v>
       </c>
       <c r="I28" t="n">
-        <v>-0.09</v>
+        <v>0.27</v>
       </c>
       <c r="J28" t="n">
-        <v>109.8</v>
+        <v>106.9</v>
       </c>
       <c r="K28" t="n">
-        <v>0.3</v>
+        <v>-2.9</v>
       </c>
       <c r="L28" t="n">
-        <v>0.27</v>
+        <v>-2.64</v>
       </c>
       <c r="M28" t="n">
-        <v>106.9</v>
+        <v>107.5</v>
       </c>
       <c r="N28" t="n">
-        <v>-2.9</v>
+        <v>0.6</v>
       </c>
       <c r="O28" t="n">
-        <v>-2.64</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="P28" t="n">
-        <v>106.9</v>
+        <v>107.5</v>
       </c>
       <c r="Q28" t="n">
-        <v>-2.9</v>
+        <v>0.6</v>
       </c>
       <c r="R28" t="n">
-        <v>-2.64</v>
+        <v>0.5600000000000001</v>
       </c>
     </row>
     <row r="29">
@@ -2189,49 +2189,49 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>108.8</v>
+        <v>108.6</v>
       </c>
       <c r="E29" t="n">
-        <v>-1.6</v>
+        <v>-0.2</v>
       </c>
       <c r="F29" t="n">
-        <v>-1.45</v>
+        <v>-0.18</v>
       </c>
       <c r="G29" t="n">
-        <v>108.6</v>
+        <v>106.3</v>
       </c>
       <c r="H29" t="n">
-        <v>-0.2</v>
+        <v>-2.3</v>
       </c>
       <c r="I29" t="n">
-        <v>-0.18</v>
+        <v>-2.12</v>
       </c>
       <c r="J29" t="n">
-        <v>106.3</v>
+        <v>105.5</v>
       </c>
       <c r="K29" t="n">
-        <v>-2.3</v>
+        <v>-0.8</v>
       </c>
       <c r="L29" t="n">
-        <v>-2.12</v>
+        <v>-0.75</v>
       </c>
       <c r="M29" t="n">
-        <v>105.5</v>
+        <v>106.2</v>
       </c>
       <c r="N29" t="n">
-        <v>-0.8</v>
+        <v>0.7</v>
       </c>
       <c r="O29" t="n">
-        <v>-0.75</v>
+        <v>0.66</v>
       </c>
       <c r="P29" t="n">
-        <v>105.5</v>
+        <v>106.2</v>
       </c>
       <c r="Q29" t="n">
-        <v>-0.8</v>
+        <v>0.7</v>
       </c>
       <c r="R29" t="n">
-        <v>-0.75</v>
+        <v>0.66</v>
       </c>
     </row>
     <row r="30">
@@ -2251,49 +2251,49 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>80.05</v>
+        <v>80.59999999999999</v>
       </c>
       <c r="E30" t="n">
-        <v>-1.7</v>
+        <v>0.55</v>
       </c>
       <c r="F30" t="n">
-        <v>-2.08</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="G30" t="n">
-        <v>80.59999999999999</v>
+        <v>77.8</v>
       </c>
       <c r="H30" t="n">
-        <v>0.55</v>
+        <v>-2.8</v>
       </c>
       <c r="I30" t="n">
-        <v>0.6899999999999999</v>
+        <v>-3.47</v>
       </c>
       <c r="J30" t="n">
-        <v>77.8</v>
+        <v>74.75</v>
       </c>
       <c r="K30" t="n">
-        <v>-2.8</v>
+        <v>-3.05</v>
       </c>
       <c r="L30" t="n">
-        <v>-3.47</v>
+        <v>-3.92</v>
       </c>
       <c r="M30" t="n">
-        <v>74.75</v>
+        <v>75.09999999999999</v>
       </c>
       <c r="N30" t="n">
-        <v>-3.05</v>
+        <v>0.35</v>
       </c>
       <c r="O30" t="n">
-        <v>-3.92</v>
+        <v>0.47</v>
       </c>
       <c r="P30" t="n">
-        <v>74.75</v>
+        <v>75.09999999999999</v>
       </c>
       <c r="Q30" t="n">
-        <v>-3.05</v>
+        <v>0.35</v>
       </c>
       <c r="R30" t="n">
-        <v>-3.92</v>
+        <v>0.47</v>
       </c>
     </row>
     <row r="31">
@@ -2313,49 +2313,49 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>91.40000000000001</v>
+        <v>89.55</v>
       </c>
       <c r="E31" t="n">
-        <v>-4.5</v>
+        <v>-1.85</v>
       </c>
       <c r="F31" t="n">
-        <v>-4.69</v>
+        <v>-2.02</v>
       </c>
       <c r="G31" t="n">
-        <v>89.55</v>
+        <v>92.2</v>
       </c>
       <c r="H31" t="n">
-        <v>-1.85</v>
+        <v>2.65</v>
       </c>
       <c r="I31" t="n">
-        <v>-2.02</v>
+        <v>2.96</v>
       </c>
       <c r="J31" t="n">
-        <v>92.2</v>
+        <v>89.15000000000001</v>
       </c>
       <c r="K31" t="n">
-        <v>2.65</v>
+        <v>-3.05</v>
       </c>
       <c r="L31" t="n">
-        <v>2.96</v>
+        <v>-3.31</v>
       </c>
       <c r="M31" t="n">
-        <v>89.15000000000001</v>
+        <v>89.09999999999999</v>
       </c>
       <c r="N31" t="n">
-        <v>-3.05</v>
+        <v>-0.05</v>
       </c>
       <c r="O31" t="n">
-        <v>-3.31</v>
+        <v>-0.06</v>
       </c>
       <c r="P31" t="n">
-        <v>89.15000000000001</v>
+        <v>89.09999999999999</v>
       </c>
       <c r="Q31" t="n">
-        <v>-3.05</v>
+        <v>-0.05</v>
       </c>
       <c r="R31" t="n">
-        <v>-3.31</v>
+        <v>-0.06</v>
       </c>
     </row>
     <row r="32">
@@ -2375,49 +2375,49 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>68.3</v>
+        <v>65.34999999999999</v>
       </c>
       <c r="E32" t="n">
-        <v>1.1</v>
+        <v>-2.95</v>
       </c>
       <c r="F32" t="n">
-        <v>1.64</v>
+        <v>-4.32</v>
       </c>
       <c r="G32" t="n">
-        <v>65.34999999999999</v>
+        <v>65</v>
       </c>
       <c r="H32" t="n">
-        <v>-2.95</v>
+        <v>-0.35</v>
       </c>
       <c r="I32" t="n">
-        <v>-4.32</v>
+        <v>-0.54</v>
       </c>
       <c r="J32" t="n">
-        <v>65</v>
+        <v>63.45</v>
       </c>
       <c r="K32" t="n">
-        <v>-0.35</v>
+        <v>-1.55</v>
       </c>
       <c r="L32" t="n">
-        <v>-0.54</v>
+        <v>-2.38</v>
       </c>
       <c r="M32" t="n">
-        <v>63.45</v>
+        <v>63.15</v>
       </c>
       <c r="N32" t="n">
-        <v>-1.55</v>
+        <v>-0.3</v>
       </c>
       <c r="O32" t="n">
-        <v>-2.38</v>
+        <v>-0.47</v>
       </c>
       <c r="P32" t="n">
-        <v>63.45</v>
+        <v>63.15</v>
       </c>
       <c r="Q32" t="n">
-        <v>-1.55</v>
+        <v>-0.3</v>
       </c>
       <c r="R32" t="n">
-        <v>-2.38</v>
+        <v>-0.47</v>
       </c>
     </row>
     <row r="33">
@@ -2437,49 +2437,49 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>84.5</v>
+        <v>83.84999999999999</v>
       </c>
       <c r="E33" t="n">
-        <v>-1.65</v>
+        <v>-0.65</v>
       </c>
       <c r="F33" t="n">
-        <v>-1.92</v>
+        <v>-0.77</v>
       </c>
       <c r="G33" t="n">
-        <v>83.84999999999999</v>
+        <v>81.8</v>
       </c>
       <c r="H33" t="n">
-        <v>-0.65</v>
+        <v>-2.05</v>
       </c>
       <c r="I33" t="n">
-        <v>-0.77</v>
+        <v>-2.44</v>
       </c>
       <c r="J33" t="n">
-        <v>81.8</v>
+        <v>79.55</v>
       </c>
       <c r="K33" t="n">
-        <v>-2.05</v>
+        <v>-2.25</v>
       </c>
       <c r="L33" t="n">
-        <v>-2.44</v>
+        <v>-2.75</v>
       </c>
       <c r="M33" t="n">
-        <v>79.55</v>
+        <v>79.84999999999999</v>
       </c>
       <c r="N33" t="n">
-        <v>-2.25</v>
+        <v>0.3</v>
       </c>
       <c r="O33" t="n">
-        <v>-2.75</v>
+        <v>0.38</v>
       </c>
       <c r="P33" t="n">
-        <v>79.55</v>
+        <v>79.84999999999999</v>
       </c>
       <c r="Q33" t="n">
-        <v>-2.25</v>
+        <v>0.3</v>
       </c>
       <c r="R33" t="n">
-        <v>-2.75</v>
+        <v>0.38</v>
       </c>
     </row>
     <row r="34">
@@ -2499,49 +2499,49 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>33.98</v>
+        <v>33.04</v>
       </c>
       <c r="E34" t="n">
-        <v>0.32</v>
+        <v>-0.9399999999999999</v>
       </c>
       <c r="F34" t="n">
-        <v>0.95</v>
+        <v>-2.77</v>
       </c>
       <c r="G34" t="n">
-        <v>33.04</v>
+        <v>32.32</v>
       </c>
       <c r="H34" t="n">
-        <v>-0.9399999999999999</v>
+        <v>-0.72</v>
       </c>
       <c r="I34" t="n">
-        <v>-2.77</v>
+        <v>-2.18</v>
       </c>
       <c r="J34" t="n">
-        <v>32.32</v>
+        <v>31.66</v>
       </c>
       <c r="K34" t="n">
-        <v>-0.72</v>
+        <v>-0.66</v>
       </c>
       <c r="L34" t="n">
-        <v>-2.18</v>
+        <v>-2.04</v>
       </c>
       <c r="M34" t="n">
-        <v>31.66</v>
+        <v>31.26</v>
       </c>
       <c r="N34" t="n">
-        <v>-0.66</v>
+        <v>-0.4</v>
       </c>
       <c r="O34" t="n">
-        <v>-2.04</v>
+        <v>-1.26</v>
       </c>
       <c r="P34" t="n">
-        <v>31.66</v>
+        <v>31.26</v>
       </c>
       <c r="Q34" t="n">
-        <v>-0.66</v>
+        <v>-0.4</v>
       </c>
       <c r="R34" t="n">
-        <v>-2.04</v>
+        <v>-1.26</v>
       </c>
     </row>
     <row r="35">
@@ -2561,49 +2561,49 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>4.44</v>
+        <v>4.37</v>
       </c>
       <c r="E35" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="F35" t="n">
+        <v>-1.58</v>
+      </c>
+      <c r="G35" t="n">
+        <v>4.33</v>
+      </c>
+      <c r="H35" t="n">
         <v>-0.04</v>
       </c>
-      <c r="F35" t="n">
-        <v>-0.89</v>
-      </c>
-      <c r="G35" t="n">
-        <v>4.37</v>
-      </c>
-      <c r="H35" t="n">
-        <v>-0.07000000000000001</v>
-      </c>
       <c r="I35" t="n">
-        <v>-1.58</v>
+        <v>-0.92</v>
       </c>
       <c r="J35" t="n">
-        <v>4.33</v>
+        <v>4.25</v>
       </c>
       <c r="K35" t="n">
-        <v>-0.04</v>
+        <v>-0.08</v>
       </c>
       <c r="L35" t="n">
-        <v>-0.92</v>
+        <v>-1.85</v>
       </c>
       <c r="M35" t="n">
-        <v>4.33</v>
+        <v>4.24</v>
       </c>
       <c r="N35" t="n">
-        <v>-0.04</v>
+        <v>-0.01</v>
       </c>
       <c r="O35" t="n">
-        <v>-0.92</v>
+        <v>-0.24</v>
       </c>
       <c r="P35" t="n">
-        <v>4.33</v>
+        <v>4.24</v>
       </c>
       <c r="Q35" t="n">
-        <v>-0.04</v>
+        <v>-0.01</v>
       </c>
       <c r="R35" t="n">
-        <v>-0.92</v>
+        <v>-0.24</v>
       </c>
     </row>
     <row r="36">
@@ -2623,49 +2623,49 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>9.56</v>
+        <v>9.41</v>
       </c>
       <c r="E36" t="n">
-        <v>-0.09</v>
+        <v>-0.15</v>
       </c>
       <c r="F36" t="n">
-        <v>-0.93</v>
+        <v>-1.57</v>
       </c>
       <c r="G36" t="n">
-        <v>9.41</v>
+        <v>9.33</v>
       </c>
       <c r="H36" t="n">
-        <v>-0.15</v>
+        <v>-0.08</v>
       </c>
       <c r="I36" t="n">
-        <v>-1.57</v>
+        <v>-0.85</v>
       </c>
       <c r="J36" t="n">
-        <v>9.33</v>
+        <v>9.140000000000001</v>
       </c>
       <c r="K36" t="n">
-        <v>-0.08</v>
+        <v>-0.19</v>
       </c>
       <c r="L36" t="n">
-        <v>-0.85</v>
+        <v>-2.04</v>
       </c>
       <c r="M36" t="n">
-        <v>9.33</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="N36" t="n">
-        <v>-0.08</v>
+        <v>-0.02</v>
       </c>
       <c r="O36" t="n">
-        <v>-0.85</v>
+        <v>-0.22</v>
       </c>
       <c r="P36" t="n">
-        <v>9.33</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="Q36" t="n">
-        <v>-0.08</v>
+        <v>-0.02</v>
       </c>
       <c r="R36" t="n">
-        <v>-0.85</v>
+        <v>-0.22</v>
       </c>
     </row>
     <row r="37">
@@ -2685,49 +2685,49 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="E37" t="n">
-        <v>-4.8</v>
+        <v>-2</v>
       </c>
       <c r="F37" t="n">
-        <v>-1.17</v>
+        <v>-0.5</v>
       </c>
       <c r="G37" t="n">
-        <v>402</v>
+        <v>400.4</v>
       </c>
       <c r="H37" t="n">
-        <v>-2</v>
+        <v>-1.6</v>
       </c>
       <c r="I37" t="n">
-        <v>-0.5</v>
+        <v>-0.4</v>
       </c>
       <c r="J37" t="n">
-        <v>400.4</v>
+        <v>397</v>
       </c>
       <c r="K37" t="n">
-        <v>-1.6</v>
+        <v>-3.4</v>
       </c>
       <c r="L37" t="n">
-        <v>-0.4</v>
+        <v>-0.85</v>
       </c>
       <c r="M37" t="n">
-        <v>397</v>
+        <v>392.6</v>
       </c>
       <c r="N37" t="n">
-        <v>-3.4</v>
+        <v>-4.4</v>
       </c>
       <c r="O37" t="n">
-        <v>-0.85</v>
+        <v>-1.11</v>
       </c>
       <c r="P37" t="n">
-        <v>397</v>
+        <v>392.6</v>
       </c>
       <c r="Q37" t="n">
-        <v>-3.4</v>
+        <v>-4.4</v>
       </c>
       <c r="R37" t="n">
-        <v>-0.85</v>
+        <v>-1.11</v>
       </c>
     </row>
     <row r="38">
@@ -2747,49 +2747,49 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>14.18</v>
+        <v>14.03</v>
       </c>
       <c r="E38" t="n">
-        <v>0.05</v>
+        <v>-0.15</v>
       </c>
       <c r="F38" t="n">
-        <v>0.35</v>
+        <v>-1.06</v>
       </c>
       <c r="G38" t="n">
-        <v>14.03</v>
+        <v>13.79</v>
       </c>
       <c r="H38" t="n">
+        <v>-0.24</v>
+      </c>
+      <c r="I38" t="n">
+        <v>-1.71</v>
+      </c>
+      <c r="J38" t="n">
+        <v>13.38</v>
+      </c>
+      <c r="K38" t="n">
+        <v>-0.41</v>
+      </c>
+      <c r="L38" t="n">
+        <v>-2.97</v>
+      </c>
+      <c r="M38" t="n">
+        <v>13.36</v>
+      </c>
+      <c r="N38" t="n">
+        <v>-0.02</v>
+      </c>
+      <c r="O38" t="n">
         <v>-0.15</v>
       </c>
-      <c r="I38" t="n">
-        <v>-1.06</v>
-      </c>
-      <c r="J38" t="n">
-        <v>13.79</v>
-      </c>
-      <c r="K38" t="n">
-        <v>-0.24</v>
-      </c>
-      <c r="L38" t="n">
-        <v>-1.71</v>
-      </c>
-      <c r="M38" t="n">
-        <v>13.38</v>
-      </c>
-      <c r="N38" t="n">
-        <v>-0.41</v>
-      </c>
-      <c r="O38" t="n">
-        <v>-2.97</v>
-      </c>
       <c r="P38" t="n">
-        <v>13.38</v>
+        <v>13.36</v>
       </c>
       <c r="Q38" t="n">
-        <v>-0.41</v>
+        <v>-0.02</v>
       </c>
       <c r="R38" t="n">
-        <v>-2.97</v>
+        <v>-0.15</v>
       </c>
     </row>
     <row r="39">
@@ -2809,49 +2809,49 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>572.5</v>
+        <v>562</v>
       </c>
       <c r="E39" t="n">
-        <v>-2</v>
+        <v>-10.5</v>
       </c>
       <c r="F39" t="n">
-        <v>-0.35</v>
+        <v>-1.83</v>
       </c>
       <c r="G39" t="n">
         <v>562</v>
       </c>
       <c r="H39" t="n">
-        <v>-10.5</v>
+        <v>0</v>
       </c>
       <c r="I39" t="n">
-        <v>-1.83</v>
+        <v>0</v>
       </c>
       <c r="J39" t="n">
-        <v>562</v>
+        <v>561.5</v>
       </c>
       <c r="K39" t="n">
-        <v>0</v>
+        <v>-0.5</v>
       </c>
       <c r="L39" t="n">
-        <v>0</v>
+        <v>-0.09</v>
       </c>
       <c r="M39" t="n">
-        <v>561.5</v>
+        <v>547.5</v>
       </c>
       <c r="N39" t="n">
-        <v>-0.5</v>
+        <v>-14</v>
       </c>
       <c r="O39" t="n">
-        <v>-0.09</v>
+        <v>-2.49</v>
       </c>
       <c r="P39" t="n">
-        <v>561.5</v>
+        <v>547.5</v>
       </c>
       <c r="Q39" t="n">
-        <v>-0.5</v>
+        <v>-14</v>
       </c>
       <c r="R39" t="n">
-        <v>-0.09</v>
+        <v>-2.49</v>
       </c>
     </row>
     <row r="40">
@@ -2871,49 +2871,49 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>42</v>
+        <v>42.38</v>
       </c>
       <c r="E40" t="n">
-        <v>-1.4</v>
+        <v>0.38</v>
       </c>
       <c r="F40" t="n">
-        <v>-3.23</v>
+        <v>0.9</v>
       </c>
       <c r="G40" t="n">
-        <v>42.38</v>
+        <v>42.3</v>
       </c>
       <c r="H40" t="n">
-        <v>0.38</v>
+        <v>-0.08</v>
       </c>
       <c r="I40" t="n">
-        <v>0.9</v>
+        <v>-0.19</v>
       </c>
       <c r="J40" t="n">
-        <v>42.3</v>
+        <v>41.6</v>
       </c>
       <c r="K40" t="n">
-        <v>-0.08</v>
+        <v>-0.7</v>
       </c>
       <c r="L40" t="n">
-        <v>-0.19</v>
+        <v>-1.65</v>
       </c>
       <c r="M40" t="n">
-        <v>41.6</v>
+        <v>41.34</v>
       </c>
       <c r="N40" t="n">
-        <v>-0.7</v>
+        <v>-0.26</v>
       </c>
       <c r="O40" t="n">
-        <v>-1.65</v>
+        <v>-0.62</v>
       </c>
       <c r="P40" t="n">
-        <v>41.6</v>
+        <v>41.34</v>
       </c>
       <c r="Q40" t="n">
-        <v>-0.7</v>
+        <v>-0.26</v>
       </c>
       <c r="R40" t="n">
-        <v>-1.65</v>
+        <v>-0.62</v>
       </c>
     </row>
     <row r="41">
@@ -2933,49 +2933,49 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>31.88</v>
+        <v>31.7</v>
       </c>
       <c r="E41" t="n">
-        <v>-0.39</v>
+        <v>-0.18</v>
       </c>
       <c r="F41" t="n">
-        <v>-1.21</v>
+        <v>-0.5600000000000001</v>
       </c>
       <c r="G41" t="n">
-        <v>31.7</v>
+        <v>31.35</v>
       </c>
       <c r="H41" t="n">
-        <v>-0.18</v>
+        <v>-0.35</v>
       </c>
       <c r="I41" t="n">
-        <v>-0.5600000000000001</v>
+        <v>-1.1</v>
       </c>
       <c r="J41" t="n">
-        <v>31.35</v>
+        <v>31.39</v>
       </c>
       <c r="K41" t="n">
-        <v>-0.35</v>
+        <v>0.04</v>
       </c>
       <c r="L41" t="n">
-        <v>-1.1</v>
+        <v>0.13</v>
       </c>
       <c r="M41" t="n">
-        <v>31.39</v>
+        <v>31.6</v>
       </c>
       <c r="N41" t="n">
-        <v>0.04</v>
+        <v>0.21</v>
       </c>
       <c r="O41" t="n">
-        <v>0.13</v>
+        <v>0.67</v>
       </c>
       <c r="P41" t="n">
-        <v>31.39</v>
+        <v>31.6</v>
       </c>
       <c r="Q41" t="n">
-        <v>0.04</v>
+        <v>0.21</v>
       </c>
       <c r="R41" t="n">
-        <v>0.13</v>
+        <v>0.67</v>
       </c>
     </row>
     <row r="42">
@@ -2995,49 +2995,49 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>78.47</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="E42" t="n">
-        <v>-0.18</v>
+        <v>-0.37</v>
       </c>
       <c r="F42" t="n">
-        <v>-0.23</v>
+        <v>-0.47</v>
       </c>
       <c r="G42" t="n">
-        <v>78.09999999999999</v>
+        <v>77.5</v>
       </c>
       <c r="H42" t="n">
-        <v>-0.37</v>
+        <v>-0.6</v>
       </c>
       <c r="I42" t="n">
-        <v>-0.47</v>
+        <v>-0.77</v>
       </c>
       <c r="J42" t="n">
-        <v>77.5</v>
+        <v>76.79000000000001</v>
       </c>
       <c r="K42" t="n">
-        <v>-0.6</v>
+        <v>-0.71</v>
       </c>
       <c r="L42" t="n">
-        <v>-0.77</v>
+        <v>-0.92</v>
       </c>
       <c r="M42" t="n">
-        <v>76.79000000000001</v>
+        <v>77</v>
       </c>
       <c r="N42" t="n">
-        <v>-0.71</v>
+        <v>0.21</v>
       </c>
       <c r="O42" t="n">
-        <v>-0.92</v>
+        <v>0.27</v>
       </c>
       <c r="P42" t="n">
-        <v>76.79000000000001</v>
+        <v>77</v>
       </c>
       <c r="Q42" t="n">
-        <v>-0.71</v>
+        <v>0.21</v>
       </c>
       <c r="R42" t="n">
-        <v>-0.92</v>
+        <v>0.27</v>
       </c>
     </row>
     <row r="43">
@@ -3057,49 +3057,49 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>41.75</v>
+        <v>41.6</v>
       </c>
       <c r="E43" t="n">
-        <v>-0.26</v>
+        <v>-0.15</v>
       </c>
       <c r="F43" t="n">
-        <v>-0.62</v>
+        <v>-0.36</v>
       </c>
       <c r="G43" t="n">
-        <v>41.6</v>
+        <v>41.18</v>
       </c>
       <c r="H43" t="n">
-        <v>-0.15</v>
+        <v>-0.42</v>
       </c>
       <c r="I43" t="n">
-        <v>-0.36</v>
+        <v>-1.01</v>
       </c>
       <c r="J43" t="n">
-        <v>41.18</v>
+        <v>40.99</v>
       </c>
       <c r="K43" t="n">
-        <v>-0.42</v>
+        <v>-0.19</v>
       </c>
       <c r="L43" t="n">
-        <v>-1.01</v>
+        <v>-0.46</v>
       </c>
       <c r="M43" t="n">
-        <v>40.99</v>
+        <v>41.26</v>
       </c>
       <c r="N43" t="n">
-        <v>-0.19</v>
+        <v>0.27</v>
       </c>
       <c r="O43" t="n">
-        <v>-0.46</v>
+        <v>0.66</v>
       </c>
       <c r="P43" t="n">
-        <v>40.99</v>
+        <v>41.26</v>
       </c>
       <c r="Q43" t="n">
-        <v>-0.19</v>
+        <v>0.27</v>
       </c>
       <c r="R43" t="n">
-        <v>-0.46</v>
+        <v>0.66</v>
       </c>
     </row>
     <row r="44">
@@ -3119,49 +3119,49 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>6.11</v>
+        <v>6.21</v>
       </c>
       <c r="E44" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="F44" t="n">
-        <v>0</v>
+        <v>1.64</v>
       </c>
       <c r="G44" t="n">
-        <v>6.21</v>
+        <v>6.19</v>
       </c>
       <c r="H44" t="n">
-        <v>0.1</v>
+        <v>-0.02</v>
       </c>
       <c r="I44" t="n">
-        <v>1.64</v>
+        <v>-0.32</v>
       </c>
       <c r="J44" t="n">
-        <v>6.19</v>
+        <v>6.1</v>
       </c>
       <c r="K44" t="n">
-        <v>-0.02</v>
+        <v>-0.09</v>
       </c>
       <c r="L44" t="n">
-        <v>-0.32</v>
+        <v>-1.45</v>
       </c>
       <c r="M44" t="n">
         <v>6.1</v>
       </c>
       <c r="N44" t="n">
-        <v>-0.09</v>
+        <v>0</v>
       </c>
       <c r="O44" t="n">
-        <v>-1.45</v>
+        <v>0</v>
       </c>
       <c r="P44" t="n">
         <v>6.1</v>
       </c>
       <c r="Q44" t="n">
-        <v>-0.09</v>
+        <v>0</v>
       </c>
       <c r="R44" t="n">
-        <v>-1.45</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45">
@@ -3181,49 +3181,49 @@
         </is>
       </c>
       <c r="D45" t="n">
+        <v>2.19</v>
+      </c>
+      <c r="E45" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="F45" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="G45" t="n">
         <v>2.17</v>
       </c>
-      <c r="E45" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="F45" t="n">
-        <v>0.46</v>
-      </c>
-      <c r="G45" t="n">
-        <v>2.19</v>
-      </c>
       <c r="H45" t="n">
-        <v>0.02</v>
+        <v>-0.02</v>
       </c>
       <c r="I45" t="n">
-        <v>0.92</v>
+        <v>-0.91</v>
       </c>
       <c r="J45" t="n">
-        <v>2.17</v>
+        <v>2.15</v>
       </c>
       <c r="K45" t="n">
         <v>-0.02</v>
       </c>
       <c r="L45" t="n">
-        <v>-0.91</v>
+        <v>-0.92</v>
       </c>
       <c r="M45" t="n">
         <v>2.15</v>
       </c>
       <c r="N45" t="n">
-        <v>-0.02</v>
+        <v>0</v>
       </c>
       <c r="O45" t="n">
-        <v>-0.92</v>
+        <v>0</v>
       </c>
       <c r="P45" t="n">
         <v>2.15</v>
       </c>
       <c r="Q45" t="n">
-        <v>-0.02</v>
+        <v>0</v>
       </c>
       <c r="R45" t="n">
-        <v>-0.92</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46">
@@ -3243,49 +3243,49 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>3.97</v>
+        <v>4.06</v>
       </c>
       <c r="E46" t="n">
         <v>0.09</v>
       </c>
       <c r="F46" t="n">
-        <v>2.32</v>
+        <v>2.27</v>
       </c>
       <c r="G46" t="n">
-        <v>4.06</v>
+        <v>4</v>
       </c>
       <c r="H46" t="n">
-        <v>0.09</v>
+        <v>-0.06</v>
       </c>
       <c r="I46" t="n">
-        <v>2.27</v>
+        <v>-1.48</v>
       </c>
       <c r="J46" t="n">
-        <v>4</v>
+        <v>3.93</v>
       </c>
       <c r="K46" t="n">
-        <v>-0.06</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="L46" t="n">
-        <v>-1.48</v>
+        <v>-1.75</v>
       </c>
       <c r="M46" t="n">
-        <v>3.93</v>
+        <v>3.91</v>
       </c>
       <c r="N46" t="n">
-        <v>-0.07000000000000001</v>
+        <v>-0.02</v>
       </c>
       <c r="O46" t="n">
-        <v>-1.75</v>
+        <v>-0.51</v>
       </c>
       <c r="P46" t="n">
-        <v>3.93</v>
+        <v>3.91</v>
       </c>
       <c r="Q46" t="n">
-        <v>-0.07000000000000001</v>
+        <v>-0.02</v>
       </c>
       <c r="R46" t="n">
-        <v>-1.75</v>
+        <v>-0.51</v>
       </c>
     </row>
     <row r="47">
@@ -3305,49 +3305,49 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>10.4</v>
+        <v>10.34</v>
       </c>
       <c r="E47" t="n">
-        <v>-0.08</v>
+        <v>-0.06</v>
       </c>
       <c r="F47" t="n">
-        <v>-0.76</v>
+        <v>-0.58</v>
       </c>
       <c r="G47" t="n">
-        <v>10.34</v>
+        <v>10.37</v>
       </c>
       <c r="H47" t="n">
-        <v>-0.06</v>
+        <v>0.03</v>
       </c>
       <c r="I47" t="n">
-        <v>-0.58</v>
+        <v>0.29</v>
       </c>
       <c r="J47" t="n">
-        <v>10.37</v>
+        <v>10.27</v>
       </c>
       <c r="K47" t="n">
-        <v>0.03</v>
+        <v>-0.1</v>
       </c>
       <c r="L47" t="n">
-        <v>0.29</v>
+        <v>-0.96</v>
       </c>
       <c r="M47" t="n">
-        <v>10.27</v>
+        <v>10.24</v>
       </c>
       <c r="N47" t="n">
-        <v>-0.1</v>
+        <v>-0.03</v>
       </c>
       <c r="O47" t="n">
-        <v>-0.96</v>
+        <v>-0.29</v>
       </c>
       <c r="P47" t="n">
-        <v>10.27</v>
+        <v>10.24</v>
       </c>
       <c r="Q47" t="n">
-        <v>-0.1</v>
+        <v>-0.03</v>
       </c>
       <c r="R47" t="n">
-        <v>-0.96</v>
+        <v>-0.29</v>
       </c>
     </row>
     <row r="48">
@@ -3367,49 +3367,49 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>0.33</v>
+        <v>0.34</v>
       </c>
       <c r="E48" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="F48" t="n">
+        <v>3.03</v>
+      </c>
+      <c r="G48" t="n">
+        <v>0.335</v>
+      </c>
+      <c r="H48" t="n">
         <v>-0.005</v>
       </c>
-      <c r="F48" t="n">
-        <v>-1.49</v>
-      </c>
-      <c r="G48" t="n">
-        <v>0.34</v>
-      </c>
-      <c r="H48" t="n">
-        <v>0.01</v>
-      </c>
       <c r="I48" t="n">
-        <v>3.03</v>
+        <v>-1.47</v>
       </c>
       <c r="J48" t="n">
-        <v>0.335</v>
+        <v>0.325</v>
       </c>
       <c r="K48" t="n">
+        <v>-0.01</v>
+      </c>
+      <c r="L48" t="n">
+        <v>-2.99</v>
+      </c>
+      <c r="M48" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="N48" t="n">
         <v>-0.005</v>
       </c>
-      <c r="L48" t="n">
-        <v>-1.47</v>
-      </c>
-      <c r="M48" t="n">
-        <v>0.325</v>
-      </c>
-      <c r="N48" t="n">
-        <v>-0.01</v>
-      </c>
       <c r="O48" t="n">
-        <v>-2.99</v>
+        <v>-1.54</v>
       </c>
       <c r="P48" t="n">
-        <v>0.325</v>
+        <v>0.32</v>
       </c>
       <c r="Q48" t="n">
-        <v>-0.01</v>
+        <v>-0.005</v>
       </c>
       <c r="R48" t="n">
-        <v>-2.99</v>
+        <v>-1.54</v>
       </c>
     </row>
     <row r="49">
@@ -3429,49 +3429,49 @@
         </is>
       </c>
       <c r="D49" t="n">
+        <v>4.54</v>
+      </c>
+      <c r="E49" t="n">
+        <v>-0.02</v>
+      </c>
+      <c r="F49" t="n">
+        <v>-0.44</v>
+      </c>
+      <c r="G49" t="n">
         <v>4.56</v>
       </c>
-      <c r="E49" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="F49" t="n">
-        <v>0.88</v>
-      </c>
-      <c r="G49" t="n">
-        <v>4.54</v>
-      </c>
       <c r="H49" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="I49" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="J49" t="n">
+        <v>4.52</v>
+      </c>
+      <c r="K49" t="n">
+        <v>-0.04</v>
+      </c>
+      <c r="L49" t="n">
+        <v>-0.88</v>
+      </c>
+      <c r="M49" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="N49" t="n">
         <v>-0.02</v>
       </c>
-      <c r="I49" t="n">
+      <c r="O49" t="n">
         <v>-0.44</v>
       </c>
-      <c r="J49" t="n">
-        <v>4.56</v>
-      </c>
-      <c r="K49" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="L49" t="n">
-        <v>0.44</v>
-      </c>
-      <c r="M49" t="n">
-        <v>4.52</v>
-      </c>
-      <c r="N49" t="n">
-        <v>-0.04</v>
-      </c>
-      <c r="O49" t="n">
-        <v>-0.88</v>
-      </c>
       <c r="P49" t="n">
-        <v>4.52</v>
+        <v>4.5</v>
       </c>
       <c r="Q49" t="n">
-        <v>-0.04</v>
+        <v>-0.02</v>
       </c>
       <c r="R49" t="n">
-        <v>-0.88</v>
+        <v>-0.44</v>
       </c>
     </row>
     <row r="50">
@@ -3491,49 +3491,49 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>1.12</v>
+        <v>1.11</v>
       </c>
       <c r="E50" t="n">
         <v>-0.01</v>
       </c>
       <c r="F50" t="n">
-        <v>-0.88</v>
+        <v>-0.89</v>
       </c>
       <c r="G50" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="H50" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I50" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="J50" t="n">
         <v>1.11</v>
       </c>
-      <c r="H50" t="n">
+      <c r="K50" t="n">
         <v>-0.01</v>
       </c>
-      <c r="I50" t="n">
+      <c r="L50" t="n">
         <v>-0.89</v>
       </c>
-      <c r="J50" t="n">
-        <v>1.12</v>
-      </c>
-      <c r="K50" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="L50" t="n">
-        <v>0.9</v>
-      </c>
       <c r="M50" t="n">
-        <v>1.11</v>
+        <v>1.09</v>
       </c>
       <c r="N50" t="n">
-        <v>-0.01</v>
+        <v>-0.02</v>
       </c>
       <c r="O50" t="n">
-        <v>-0.89</v>
+        <v>-1.8</v>
       </c>
       <c r="P50" t="n">
-        <v>1.11</v>
+        <v>1.09</v>
       </c>
       <c r="Q50" t="n">
-        <v>-0.01</v>
+        <v>-0.02</v>
       </c>
       <c r="R50" t="n">
-        <v>-0.89</v>
+        <v>-1.8</v>
       </c>
     </row>
     <row r="51">
@@ -3553,49 +3553,49 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>4.94</v>
+        <v>5.14</v>
       </c>
       <c r="E51" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="F51" t="n">
-        <v>0</v>
+        <v>4.05</v>
       </c>
       <c r="G51" t="n">
-        <v>5.14</v>
+        <v>5.12</v>
       </c>
       <c r="H51" t="n">
-        <v>0.2</v>
+        <v>-0.02</v>
       </c>
       <c r="I51" t="n">
-        <v>4.05</v>
+        <v>-0.39</v>
       </c>
       <c r="J51" t="n">
-        <v>5.12</v>
+        <v>5</v>
       </c>
       <c r="K51" t="n">
+        <v>-0.12</v>
+      </c>
+      <c r="L51" t="n">
+        <v>-2.34</v>
+      </c>
+      <c r="M51" t="n">
+        <v>4.98</v>
+      </c>
+      <c r="N51" t="n">
         <v>-0.02</v>
       </c>
-      <c r="L51" t="n">
-        <v>-0.39</v>
-      </c>
-      <c r="M51" t="n">
-        <v>5</v>
-      </c>
-      <c r="N51" t="n">
-        <v>-0.12</v>
-      </c>
       <c r="O51" t="n">
-        <v>-2.34</v>
+        <v>-0.4</v>
       </c>
       <c r="P51" t="n">
-        <v>5</v>
+        <v>4.98</v>
       </c>
       <c r="Q51" t="n">
-        <v>-0.12</v>
+        <v>-0.02</v>
       </c>
       <c r="R51" t="n">
-        <v>-2.34</v>
+        <v>-0.4</v>
       </c>
     </row>
     <row r="52">
@@ -3615,49 +3615,49 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>11.79</v>
+        <v>11.88</v>
       </c>
       <c r="E52" t="n">
-        <v>0.25</v>
+        <v>0.09</v>
       </c>
       <c r="F52" t="n">
-        <v>2.17</v>
+        <v>0.76</v>
       </c>
       <c r="G52" t="n">
-        <v>11.88</v>
+        <v>11.8</v>
       </c>
       <c r="H52" t="n">
-        <v>0.09</v>
+        <v>-0.08</v>
       </c>
       <c r="I52" t="n">
-        <v>0.76</v>
+        <v>-0.67</v>
       </c>
       <c r="J52" t="n">
-        <v>11.8</v>
+        <v>11.47</v>
       </c>
       <c r="K52" t="n">
-        <v>-0.08</v>
+        <v>-0.33</v>
       </c>
       <c r="L52" t="n">
-        <v>-0.67</v>
+        <v>-2.8</v>
       </c>
       <c r="M52" t="n">
-        <v>11.47</v>
+        <v>11.43</v>
       </c>
       <c r="N52" t="n">
-        <v>-0.33</v>
+        <v>-0.04</v>
       </c>
       <c r="O52" t="n">
-        <v>-2.8</v>
+        <v>-0.35</v>
       </c>
       <c r="P52" t="n">
-        <v>11.47</v>
+        <v>11.43</v>
       </c>
       <c r="Q52" t="n">
-        <v>-0.33</v>
+        <v>-0.04</v>
       </c>
       <c r="R52" t="n">
-        <v>-2.8</v>
+        <v>-0.35</v>
       </c>
     </row>
     <row r="53">
@@ -3677,49 +3677,49 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>8.6</v>
+        <v>8.390000000000001</v>
       </c>
       <c r="E53" t="n">
-        <v>0</v>
+        <v>-0.21</v>
       </c>
       <c r="F53" t="n">
-        <v>0</v>
+        <v>-2.44</v>
       </c>
       <c r="G53" t="n">
-        <v>8.390000000000001</v>
+        <v>8.35</v>
       </c>
       <c r="H53" t="n">
-        <v>-0.21</v>
+        <v>-0.04</v>
       </c>
       <c r="I53" t="n">
-        <v>-2.44</v>
+        <v>-0.48</v>
       </c>
       <c r="J53" t="n">
-        <v>8.35</v>
+        <v>8.220000000000001</v>
       </c>
       <c r="K53" t="n">
-        <v>-0.04</v>
+        <v>-0.13</v>
       </c>
       <c r="L53" t="n">
-        <v>-0.48</v>
+        <v>-1.56</v>
       </c>
       <c r="M53" t="n">
-        <v>8.220000000000001</v>
+        <v>8.16</v>
       </c>
       <c r="N53" t="n">
-        <v>-0.13</v>
+        <v>-0.06</v>
       </c>
       <c r="O53" t="n">
-        <v>-1.56</v>
+        <v>-0.73</v>
       </c>
       <c r="P53" t="n">
-        <v>8.220000000000001</v>
+        <v>8.16</v>
       </c>
       <c r="Q53" t="n">
-        <v>-0.13</v>
+        <v>-0.06</v>
       </c>
       <c r="R53" t="n">
-        <v>-1.56</v>
+        <v>-0.73</v>
       </c>
     </row>
     <row r="54">
@@ -3748,40 +3748,40 @@
         <v>0</v>
       </c>
       <c r="G54" t="n">
-        <v>0.45</v>
+        <v>0.445</v>
       </c>
       <c r="H54" t="n">
-        <v>0</v>
+        <v>-0.005</v>
       </c>
       <c r="I54" t="n">
-        <v>0</v>
+        <v>-1.11</v>
       </c>
       <c r="J54" t="n">
         <v>0.445</v>
       </c>
       <c r="K54" t="n">
+        <v>0</v>
+      </c>
+      <c r="L54" t="n">
+        <v>0</v>
+      </c>
+      <c r="M54" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="N54" t="n">
         <v>-0.005</v>
       </c>
-      <c r="L54" t="n">
-        <v>-1.11</v>
-      </c>
-      <c r="M54" t="n">
-        <v>0.445</v>
-      </c>
-      <c r="N54" t="n">
-        <v>0</v>
-      </c>
       <c r="O54" t="n">
-        <v>0</v>
+        <v>-1.12</v>
       </c>
       <c r="P54" t="n">
-        <v>0.445</v>
+        <v>0.44</v>
       </c>
       <c r="Q54" t="n">
-        <v>0</v>
+        <v>-0.005</v>
       </c>
       <c r="R54" t="n">
-        <v>0</v>
+        <v>-1.12</v>
       </c>
     </row>
     <row r="55">
@@ -3801,31 +3801,31 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>0.625</v>
+        <v>0.62</v>
       </c>
       <c r="E55" t="n">
-        <v>0.005</v>
+        <v>-0.005</v>
       </c>
       <c r="F55" t="n">
-        <v>0.8100000000000001</v>
+        <v>-0.8</v>
       </c>
       <c r="G55" t="n">
-        <v>0.62</v>
+        <v>0.615</v>
       </c>
       <c r="H55" t="n">
         <v>-0.005</v>
       </c>
       <c r="I55" t="n">
-        <v>-0.8</v>
+        <v>-0.8100000000000001</v>
       </c>
       <c r="J55" t="n">
         <v>0.615</v>
       </c>
       <c r="K55" t="n">
-        <v>-0.005</v>
+        <v>0</v>
       </c>
       <c r="L55" t="n">
-        <v>-0.8100000000000001</v>
+        <v>0</v>
       </c>
       <c r="M55" t="n">
         <v>0.615</v>
@@ -3881,31 +3881,31 @@
         <v>0</v>
       </c>
       <c r="J56" t="n">
-        <v>0.415</v>
+        <v>0.41</v>
       </c>
       <c r="K56" t="n">
-        <v>0</v>
+        <v>-0.005</v>
       </c>
       <c r="L56" t="n">
-        <v>0</v>
+        <v>-1.2</v>
       </c>
       <c r="M56" t="n">
         <v>0.41</v>
       </c>
       <c r="N56" t="n">
-        <v>-0.005</v>
+        <v>0</v>
       </c>
       <c r="O56" t="n">
-        <v>-1.2</v>
+        <v>0</v>
       </c>
       <c r="P56" t="n">
         <v>0.41</v>
       </c>
       <c r="Q56" t="n">
-        <v>-0.005</v>
+        <v>0</v>
       </c>
       <c r="R56" t="n">
-        <v>-1.2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="57">
@@ -3925,49 +3925,49 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>3.8</v>
+        <v>3.73</v>
       </c>
       <c r="E57" t="n">
-        <v>-0.02</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="F57" t="n">
-        <v>-0.52</v>
+        <v>-1.84</v>
       </c>
       <c r="G57" t="n">
         <v>3.73</v>
       </c>
       <c r="H57" t="n">
-        <v>-0.07000000000000001</v>
+        <v>0</v>
       </c>
       <c r="I57" t="n">
-        <v>-1.84</v>
+        <v>0</v>
       </c>
       <c r="J57" t="n">
-        <v>3.73</v>
+        <v>3.71</v>
       </c>
       <c r="K57" t="n">
-        <v>0</v>
+        <v>-0.02</v>
       </c>
       <c r="L57" t="n">
-        <v>0</v>
+        <v>-0.54</v>
       </c>
       <c r="M57" t="n">
         <v>3.71</v>
       </c>
       <c r="N57" t="n">
-        <v>-0.02</v>
+        <v>0</v>
       </c>
       <c r="O57" t="n">
-        <v>-0.54</v>
+        <v>0</v>
       </c>
       <c r="P57" t="n">
         <v>3.71</v>
       </c>
       <c r="Q57" t="n">
-        <v>-0.02</v>
+        <v>0</v>
       </c>
       <c r="R57" t="n">
-        <v>-0.54</v>
+        <v>0</v>
       </c>
     </row>
     <row r="58">
@@ -3987,49 +3987,49 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>0.077</v>
+        <v>0.075</v>
       </c>
       <c r="E58" t="n">
-        <v>0</v>
+        <v>-0.002</v>
       </c>
       <c r="F58" t="n">
-        <v>0</v>
+        <v>-2.6</v>
       </c>
       <c r="G58" t="n">
-        <v>0.075</v>
+        <v>0.076</v>
       </c>
       <c r="H58" t="n">
-        <v>-0.002</v>
+        <v>0.001</v>
       </c>
       <c r="I58" t="n">
-        <v>-2.6</v>
+        <v>1.33</v>
       </c>
       <c r="J58" t="n">
         <v>0.076</v>
       </c>
       <c r="K58" t="n">
+        <v>0</v>
+      </c>
+      <c r="L58" t="n">
+        <v>0</v>
+      </c>
+      <c r="M58" t="n">
+        <v>0.077</v>
+      </c>
+      <c r="N58" t="n">
         <v>0.001</v>
       </c>
-      <c r="L58" t="n">
-        <v>1.33</v>
-      </c>
-      <c r="M58" t="n">
-        <v>0.076</v>
-      </c>
-      <c r="N58" t="n">
-        <v>0</v>
-      </c>
       <c r="O58" t="n">
-        <v>0</v>
+        <v>1.32</v>
       </c>
       <c r="P58" t="n">
-        <v>0.076</v>
+        <v>0.077</v>
       </c>
       <c r="Q58" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="R58" t="n">
-        <v>0</v>
+        <v>1.32</v>
       </c>
     </row>
     <row r="59">
@@ -4049,49 +4049,49 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>25.13</v>
+        <v>24.9</v>
       </c>
       <c r="E59" t="n">
-        <v>-0.17</v>
+        <v>-0.23</v>
       </c>
       <c r="F59" t="n">
-        <v>-0.67</v>
+        <v>-0.92</v>
       </c>
       <c r="G59" t="n">
-        <v>24.9</v>
+        <v>24.78</v>
       </c>
       <c r="H59" t="n">
-        <v>-0.23</v>
+        <v>-0.12</v>
       </c>
       <c r="I59" t="n">
-        <v>-0.92</v>
+        <v>-0.48</v>
       </c>
       <c r="J59" t="n">
-        <v>24.78</v>
+        <v>24.68</v>
       </c>
       <c r="K59" t="n">
-        <v>-0.12</v>
+        <v>-0.1</v>
       </c>
       <c r="L59" t="n">
-        <v>-0.48</v>
+        <v>-0.4</v>
       </c>
       <c r="M59" t="n">
-        <v>24.68</v>
+        <v>24.3</v>
       </c>
       <c r="N59" t="n">
-        <v>-0.1</v>
+        <v>-0.38</v>
       </c>
       <c r="O59" t="n">
-        <v>-0.4</v>
+        <v>-1.54</v>
       </c>
       <c r="P59" t="n">
-        <v>24.68</v>
+        <v>24.3</v>
       </c>
       <c r="Q59" t="n">
-        <v>-0.1</v>
+        <v>-0.38</v>
       </c>
       <c r="R59" t="n">
-        <v>-0.4</v>
+        <v>-1.54</v>
       </c>
     </row>
     <row r="60">
@@ -4111,16 +4111,16 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>3.14</v>
+        <v>3.13</v>
       </c>
       <c r="E60" t="n">
-        <v>0.01</v>
+        <v>-0.01</v>
       </c>
       <c r="F60" t="n">
-        <v>0.32</v>
+        <v>-0.32</v>
       </c>
       <c r="G60" t="n">
-        <v>3.13</v>
+        <v>3.12</v>
       </c>
       <c r="H60" t="n">
         <v>-0.01</v>
@@ -4129,7 +4129,7 @@
         <v>-0.32</v>
       </c>
       <c r="J60" t="n">
-        <v>3.12</v>
+        <v>3.11</v>
       </c>
       <c r="K60" t="n">
         <v>-0.01</v>
@@ -4141,19 +4141,19 @@
         <v>3.11</v>
       </c>
       <c r="N60" t="n">
-        <v>-0.01</v>
+        <v>0</v>
       </c>
       <c r="O60" t="n">
-        <v>-0.32</v>
+        <v>0</v>
       </c>
       <c r="P60" t="n">
         <v>3.11</v>
       </c>
       <c r="Q60" t="n">
-        <v>-0.01</v>
+        <v>0</v>
       </c>
       <c r="R60" t="n">
-        <v>-0.32</v>
+        <v>0</v>
       </c>
     </row>
     <row r="61">
@@ -4173,16 +4173,16 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>0.925</v>
+        <v>0.93</v>
       </c>
       <c r="E61" t="n">
-        <v>0.01</v>
+        <v>0.005</v>
       </c>
       <c r="F61" t="n">
-        <v>1.09</v>
+        <v>0.54</v>
       </c>
       <c r="G61" t="n">
-        <v>0.93</v>
+        <v>0.9350000000000001</v>
       </c>
       <c r="H61" t="n">
         <v>0.005</v>
@@ -4191,31 +4191,31 @@
         <v>0.54</v>
       </c>
       <c r="J61" t="n">
-        <v>0.9350000000000001</v>
+        <v>0.93</v>
       </c>
       <c r="K61" t="n">
-        <v>0.005</v>
+        <v>-0.005</v>
       </c>
       <c r="L61" t="n">
-        <v>0.54</v>
+        <v>-0.53</v>
       </c>
       <c r="M61" t="n">
-        <v>0.93</v>
+        <v>0.915</v>
       </c>
       <c r="N61" t="n">
-        <v>-0.005</v>
+        <v>-0.015</v>
       </c>
       <c r="O61" t="n">
-        <v>-0.53</v>
+        <v>-1.61</v>
       </c>
       <c r="P61" t="n">
-        <v>0.93</v>
+        <v>0.915</v>
       </c>
       <c r="Q61" t="n">
-        <v>-0.005</v>
+        <v>-0.015</v>
       </c>
       <c r="R61" t="n">
-        <v>-0.53</v>
+        <v>-1.61</v>
       </c>
     </row>
   </sheetData>

</xml_diff>